<commit_message>
Dashboard update 2026-10-11 12:07
</commit_message>
<xml_diff>
--- a/excel/Investavimas Rima.xlsx
+++ b/excel/Investavimas Rima.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.08.08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81414D25-56C4-4E11-BE5D-E27F1E97A215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6581A8F-7EAC-4F3D-9925-DCD5BCB07754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2090,10 +2090,10 @@
         <v>1.835</v>
       </c>
       <c r="K8" s="21">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="L8" s="4">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="M8" s="12">
         <f t="shared" ref="M8:M11" si="35">(L8-K8)/K8</f>
@@ -2181,15 +2181,15 @@
       </c>
       <c r="AM8" s="4">
         <f t="shared" si="3"/>
-        <v>840</v>
+        <v>640</v>
       </c>
       <c r="AN8" s="4">
         <f t="shared" si="28"/>
-        <v>810</v>
+        <v>610</v>
       </c>
       <c r="AO8" s="4">
         <f t="shared" si="4"/>
-        <v>915.05</v>
+        <v>715.05</v>
       </c>
       <c r="AP8" s="4">
         <f t="shared" si="5"/>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="AQ8" s="13">
         <f t="shared" si="6"/>
-        <v>8.9345238095238047E-2</v>
+        <v>0.11726562499999993</v>
       </c>
       <c r="AR8" s="4">
         <f t="shared" si="29"/>
@@ -2210,27 +2210,27 @@
       </c>
       <c r="AU8" s="4">
         <f t="shared" si="18"/>
-        <v>1050</v>
+        <v>850</v>
       </c>
       <c r="AV8" s="4">
         <f t="shared" si="30"/>
-        <v>840</v>
+        <v>640</v>
       </c>
       <c r="AW8" s="4">
         <f t="shared" si="19"/>
-        <v>1129.6799999999998</v>
+        <v>929.68</v>
       </c>
       <c r="AX8" s="4">
         <f t="shared" si="7"/>
-        <v>79.679999999999836</v>
+        <v>79.67999999999995</v>
       </c>
       <c r="AY8" s="13">
         <f t="shared" si="8"/>
-        <v>7.5885714285714126E-2</v>
+        <v>9.3741176470588175E-2</v>
       </c>
       <c r="AZ8" s="4">
         <f t="shared" si="31"/>
-        <v>20.529999999999859</v>
+        <v>20.529999999999973</v>
       </c>
       <c r="BB8" s="8">
         <f t="shared" si="9"/>
@@ -2307,10 +2307,10 @@
         <v>1.835</v>
       </c>
       <c r="K9" s="21">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="L9" s="4">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="M9" s="12">
         <f t="shared" si="35"/>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="AM9" s="4">
         <f t="shared" si="3"/>
-        <v>1440</v>
+        <v>1240</v>
       </c>
       <c r="AN9" s="4">
         <f t="shared" si="28"/>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="AO9" s="4">
         <f t="shared" si="4"/>
-        <v>1518.75</v>
+        <v>1318.75</v>
       </c>
       <c r="AP9" s="4">
         <f t="shared" si="5"/>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="AQ9" s="13">
         <f t="shared" si="6"/>
-        <v>5.46875E-2</v>
+        <v>6.3508064516129031E-2</v>
       </c>
       <c r="AR9" s="4">
         <f t="shared" si="29"/>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="AU9" s="4">
         <f t="shared" si="18"/>
-        <v>1680</v>
+        <v>1480</v>
       </c>
       <c r="AV9" s="4">
         <f t="shared" si="30"/>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="AW9" s="4">
         <f t="shared" si="19"/>
-        <v>1764.76</v>
+        <v>1564.76</v>
       </c>
       <c r="AX9" s="4">
         <f t="shared" si="7"/>
@@ -2444,11 +2444,11 @@
       </c>
       <c r="AY9" s="13">
         <f t="shared" si="8"/>
-        <v>5.045238095238095E-2</v>
+        <v>5.7270270270270263E-2</v>
       </c>
       <c r="AZ9" s="4">
         <f t="shared" si="31"/>
-        <v>5.0800000000001546</v>
+        <v>5.0800000000000409</v>
       </c>
       <c r="BB9" s="8">
         <f t="shared" si="9"/>
@@ -2525,10 +2525,10 @@
         <v>1.835</v>
       </c>
       <c r="K10" s="21">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="L10" s="4">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="M10" s="12">
         <f t="shared" si="35"/>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="AM10" s="4">
         <f t="shared" si="3"/>
-        <v>1460</v>
+        <v>1260</v>
       </c>
       <c r="AN10" s="4">
         <f t="shared" si="28"/>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="AO10" s="4">
         <f t="shared" si="4"/>
-        <v>1570.02</v>
+        <v>1370.02</v>
       </c>
       <c r="AP10" s="4">
         <f t="shared" si="5"/>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="AQ10" s="13">
         <f t="shared" si="6"/>
-        <v>7.535616438356163E-2</v>
+        <v>8.7317460317460308E-2</v>
       </c>
       <c r="AR10" s="4">
         <f t="shared" si="29"/>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="AU10" s="4">
         <f t="shared" si="18"/>
-        <v>1730</v>
+        <v>1530</v>
       </c>
       <c r="AV10" s="4">
         <f t="shared" si="30"/>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="AW10" s="4">
         <f t="shared" si="19"/>
-        <v>1854.76</v>
+        <v>1654.76</v>
       </c>
       <c r="AX10" s="4">
         <f t="shared" si="7"/>
@@ -2661,7 +2661,7 @@
       </c>
       <c r="AY10" s="13">
         <f t="shared" si="8"/>
-        <v>7.2115606936416179E-2</v>
+        <v>8.1542483660130713E-2</v>
       </c>
       <c r="AZ10" s="4">
         <f t="shared" si="31"/>
@@ -2743,14 +2743,14 @@
         <v>1.835</v>
       </c>
       <c r="K11" s="21">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="L11" s="4">
-        <v>525</v>
+        <v>325</v>
       </c>
       <c r="M11" s="12">
         <f t="shared" si="35"/>
-        <v>0.05</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="N11" s="5">
         <v>420</v>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="AM11" s="4">
         <f t="shared" si="3"/>
-        <v>1560</v>
+        <v>1360</v>
       </c>
       <c r="AN11" s="4">
         <f t="shared" si="28"/>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="AO11" s="4">
         <f t="shared" si="4"/>
-        <v>1700.19</v>
+        <v>1500.19</v>
       </c>
       <c r="AP11" s="4">
         <f t="shared" si="5"/>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="AQ11" s="13">
         <f t="shared" si="6"/>
-        <v>8.9865384615384653E-2</v>
+        <v>0.10308088235294122</v>
       </c>
       <c r="AR11" s="4">
         <f t="shared" si="29"/>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="AU11" s="4">
         <f t="shared" si="18"/>
-        <v>1860</v>
+        <v>1660</v>
       </c>
       <c r="AV11" s="4">
         <f t="shared" si="30"/>
@@ -2871,7 +2871,7 @@
       </c>
       <c r="AW11" s="4">
         <f t="shared" si="19"/>
-        <v>2013.3000000000002</v>
+        <v>1813.3000000000002</v>
       </c>
       <c r="AX11" s="4">
         <f t="shared" si="7"/>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="AY11" s="13">
         <f t="shared" si="8"/>
-        <v>8.2419354838709769E-2</v>
+        <v>9.2349397590361551E-2</v>
       </c>
       <c r="AZ11" s="4">
         <f t="shared" si="31"/>
@@ -2961,14 +2961,14 @@
         <v>1.8366666666666664</v>
       </c>
       <c r="K12" s="21">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="L12" s="4">
-        <v>537.22</v>
+        <v>331.12</v>
       </c>
       <c r="M12" s="12">
         <f t="shared" ref="M12" si="39">(L12-K12)/K12</f>
-        <v>7.4440000000000048E-2</v>
+        <v>0.10373333333333334</v>
       </c>
       <c r="N12" s="5">
         <v>420</v>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="AM12" s="4">
         <f t="shared" si="3"/>
-        <v>1560</v>
+        <v>1360</v>
       </c>
       <c r="AN12" s="4">
         <f t="shared" si="28"/>
@@ -3060,19 +3060,19 @@
       </c>
       <c r="AO12" s="4">
         <f t="shared" si="4"/>
-        <v>1716.71</v>
+        <v>1510.6100000000001</v>
       </c>
       <c r="AP12" s="4">
         <f t="shared" si="5"/>
-        <v>156.71000000000004</v>
+        <v>150.61000000000013</v>
       </c>
       <c r="AQ12" s="13">
         <f t="shared" si="6"/>
-        <v>0.10045512820512822</v>
+        <v>0.11074264705882363</v>
       </c>
       <c r="AR12" s="4">
         <f t="shared" si="29"/>
-        <v>16.519999999999982</v>
+        <v>10.420000000000073</v>
       </c>
       <c r="AS12" s="10"/>
       <c r="AT12" s="8">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="AU12" s="4">
         <f t="shared" si="18"/>
-        <v>1860</v>
+        <v>1660</v>
       </c>
       <c r="AV12" s="4">
         <f t="shared" si="30"/>
@@ -3089,19 +3089,19 @@
       </c>
       <c r="AW12" s="4">
         <f t="shared" si="19"/>
-        <v>2034.56</v>
+        <v>1828.46</v>
       </c>
       <c r="AX12" s="4">
         <f t="shared" si="7"/>
-        <v>174.55999999999995</v>
+        <v>168.46000000000004</v>
       </c>
       <c r="AY12" s="13">
         <f t="shared" si="8"/>
-        <v>9.3849462365591371E-2</v>
+        <v>0.1014819277108434</v>
       </c>
       <c r="AZ12" s="4">
         <f t="shared" si="31"/>
-        <v>21.259999999999764</v>
+        <v>15.159999999999854</v>
       </c>
       <c r="BB12" s="8">
         <f t="shared" si="9"/>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="BF12" s="4">
         <f t="shared" si="23"/>
-        <v>12.220000000000027</v>
+        <v>6.1200000000000045</v>
       </c>
       <c r="BG12" s="4">
         <f t="shared" si="24"/>
@@ -3180,14 +3180,14 @@
         <v>1.8366666666666664</v>
       </c>
       <c r="K13" s="21">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="L13" s="4">
-        <v>537.22</v>
+        <v>331.12</v>
       </c>
       <c r="M13" s="12">
         <f t="shared" ref="M13" si="44">(L13-K13)/K13</f>
-        <v>7.4440000000000048E-2</v>
+        <v>0.10373333333333334</v>
       </c>
       <c r="N13" s="5">
         <v>420</v>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="AM13" s="4">
         <f t="shared" si="3"/>
-        <v>1560</v>
+        <v>1360</v>
       </c>
       <c r="AN13" s="4">
         <f t="shared" si="28"/>
@@ -3279,15 +3279,15 @@
       </c>
       <c r="AO13" s="4">
         <f t="shared" si="4"/>
-        <v>1721.08</v>
+        <v>1514.98</v>
       </c>
       <c r="AP13" s="4">
         <f t="shared" si="5"/>
-        <v>161.07999999999993</v>
+        <v>154.98000000000002</v>
       </c>
       <c r="AQ13" s="13">
         <f t="shared" si="6"/>
-        <v>0.10325641025641021</v>
+        <v>0.11395588235294118</v>
       </c>
       <c r="AR13" s="4">
         <f t="shared" si="29"/>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="AU13" s="4">
         <f t="shared" si="18"/>
-        <v>2020</v>
+        <v>1820</v>
       </c>
       <c r="AV13" s="4">
         <f t="shared" si="30"/>
@@ -3308,19 +3308,19 @@
       </c>
       <c r="AW13" s="4">
         <f t="shared" si="19"/>
-        <v>2206.5299999999997</v>
+        <v>2000.43</v>
       </c>
       <c r="AX13" s="4">
         <f t="shared" si="7"/>
-        <v>186.52999999999975</v>
+        <v>180.43000000000006</v>
       </c>
       <c r="AY13" s="13">
         <f t="shared" si="8"/>
-        <v>9.2341584158415715E-2</v>
+        <v>9.9137362637362669E-2</v>
       </c>
       <c r="AZ13" s="4">
         <f t="shared" si="31"/>
-        <v>11.9699999999998</v>
+        <v>11.970000000000027</v>
       </c>
       <c r="BB13" s="8">
         <f t="shared" si="9"/>
@@ -3398,14 +3398,14 @@
         <v>1.8366666666666664</v>
       </c>
       <c r="K14" s="21">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="L14" s="4">
-        <v>537.22</v>
+        <v>331.12</v>
       </c>
       <c r="M14" s="12">
         <f t="shared" ref="M14" si="50">(L14-K14)/K14</f>
-        <v>7.4440000000000048E-2</v>
+        <v>0.10373333333333334</v>
       </c>
       <c r="N14" s="5">
         <v>420</v>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="AM14" s="4">
         <f t="shared" si="3"/>
-        <v>1560</v>
+        <v>1360</v>
       </c>
       <c r="AN14" s="4">
         <f t="shared" si="28"/>
@@ -3497,15 +3497,15 @@
       </c>
       <c r="AO14" s="4">
         <f t="shared" si="4"/>
-        <v>1736.15</v>
+        <v>1530.0500000000002</v>
       </c>
       <c r="AP14" s="4">
         <f t="shared" si="5"/>
-        <v>176.15000000000009</v>
+        <v>170.05000000000018</v>
       </c>
       <c r="AQ14" s="13">
         <f t="shared" si="6"/>
-        <v>0.11291666666666672</v>
+        <v>0.12503676470588249</v>
       </c>
       <c r="AR14" s="4">
         <f t="shared" si="29"/>
@@ -3518,7 +3518,7 @@
       </c>
       <c r="AU14" s="4">
         <f t="shared" si="18"/>
-        <v>2150</v>
+        <v>1950</v>
       </c>
       <c r="AV14" s="4">
         <f t="shared" si="30"/>
@@ -3526,19 +3526,19 @@
       </c>
       <c r="AW14" s="4">
         <f t="shared" si="19"/>
-        <v>2358.63</v>
+        <v>2152.5300000000002</v>
       </c>
       <c r="AX14" s="4">
         <f t="shared" si="7"/>
-        <v>208.63000000000011</v>
+        <v>202.5300000000002</v>
       </c>
       <c r="AY14" s="13">
         <f t="shared" si="8"/>
-        <v>9.7037209302325636E-2</v>
+        <v>0.10386153846153856</v>
       </c>
       <c r="AZ14" s="4">
         <f t="shared" si="31"/>
-        <v>22.100000000000364</v>
+        <v>22.100000000000136</v>
       </c>
       <c r="BB14" s="8">
         <f t="shared" si="9"/>
@@ -3616,14 +3616,14 @@
         <v>1.8366666666666664</v>
       </c>
       <c r="K15" s="21">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="L15" s="4">
-        <v>544.55999999999995</v>
+        <v>336.24</v>
       </c>
       <c r="M15" s="12">
         <f t="shared" ref="M15" si="56">(L15-K15)/K15</f>
-        <v>8.9119999999999894E-2</v>
+        <v>0.12080000000000003</v>
       </c>
       <c r="N15" s="5">
         <v>620</v>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="AM15" s="4">
         <f t="shared" si="3"/>
-        <v>1760</v>
+        <v>1560</v>
       </c>
       <c r="AN15" s="4">
         <f t="shared" si="28"/>
@@ -3715,19 +3715,19 @@
       </c>
       <c r="AO15" s="4">
         <f t="shared" si="4"/>
-        <v>1971.55</v>
+        <v>1763.23</v>
       </c>
       <c r="AP15" s="4">
         <f t="shared" si="5"/>
-        <v>211.54999999999995</v>
+        <v>203.23000000000002</v>
       </c>
       <c r="AQ15" s="13">
         <f t="shared" si="6"/>
-        <v>0.1201988636363636</v>
+        <v>0.13027564102564104</v>
       </c>
       <c r="AR15" s="4">
         <f t="shared" si="29"/>
-        <v>35.399999999999864</v>
+        <v>33.179999999999836</v>
       </c>
       <c r="AS15" s="10"/>
       <c r="AT15" s="8">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="AU15" s="4">
         <f t="shared" si="18"/>
-        <v>2480</v>
+        <v>2280</v>
       </c>
       <c r="AV15" s="4">
         <f t="shared" si="30"/>
@@ -3744,19 +3744,19 @@
       </c>
       <c r="AW15" s="4">
         <f t="shared" si="19"/>
-        <v>2682.46</v>
+        <v>2474.1400000000003</v>
       </c>
       <c r="AX15" s="4">
         <f t="shared" si="7"/>
-        <v>202.46000000000004</v>
+        <v>194.14000000000033</v>
       </c>
       <c r="AY15" s="13">
         <f t="shared" si="8"/>
-        <v>8.1637096774193563E-2</v>
+        <v>8.5149122807017683E-2</v>
       </c>
       <c r="AZ15" s="4">
         <f t="shared" si="31"/>
-        <v>-6.1700000000000728</v>
+        <v>-8.3899999999998727</v>
       </c>
       <c r="BB15" s="8">
         <f t="shared" ref="BB15" si="63">A15</f>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="BF15" s="4">
         <f t="shared" ref="BF15" si="67">(L15-K15)-(L14-K14)</f>
-        <v>7.3399999999999181</v>
+        <v>5.1200000000000045</v>
       </c>
       <c r="BG15" s="4">
         <f t="shared" ref="BG15" si="68">(O15-N15)-(O14-N14)</f>
@@ -3834,14 +3834,14 @@
         <v>1.8366666666666664</v>
       </c>
       <c r="K16" s="21">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="L16" s="4">
-        <v>549.24</v>
+        <v>338.58</v>
       </c>
       <c r="M16" s="12">
         <f t="shared" ref="M16" si="73">(L16-K16)/K16</f>
-        <v>9.8480000000000012E-2</v>
+        <v>0.12859999999999994</v>
       </c>
       <c r="N16" s="5">
         <v>620</v>
@@ -3926,7 +3926,7 @@
       </c>
       <c r="AM16" s="4">
         <f t="shared" si="3"/>
-        <v>1800</v>
+        <v>1600</v>
       </c>
       <c r="AN16" s="4">
         <f t="shared" si="28"/>
@@ -3934,19 +3934,19 @@
       </c>
       <c r="AO16" s="4">
         <f t="shared" si="4"/>
-        <v>2028.74</v>
+        <v>1818.0799999999997</v>
       </c>
       <c r="AP16" s="4">
         <f t="shared" si="5"/>
-        <v>228.74</v>
+        <v>218.0799999999997</v>
       </c>
       <c r="AQ16" s="13">
         <f t="shared" si="6"/>
-        <v>0.12707777777777779</v>
+        <v>0.13629999999999981</v>
       </c>
       <c r="AR16" s="4">
         <f t="shared" si="29"/>
-        <v>17.190000000000055</v>
+        <v>14.849999999999682</v>
       </c>
       <c r="AS16" s="10"/>
       <c r="AT16" s="8">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="AU16" s="4">
         <f t="shared" si="18"/>
-        <v>2650</v>
+        <v>2450</v>
       </c>
       <c r="AV16" s="4">
         <f t="shared" si="30"/>
@@ -3963,19 +3963,19 @@
       </c>
       <c r="AW16" s="4">
         <f t="shared" si="19"/>
-        <v>2923.3599999999997</v>
+        <v>2712.7</v>
       </c>
       <c r="AX16" s="4">
         <f t="shared" si="7"/>
-        <v>273.35999999999967</v>
+        <v>262.69999999999982</v>
       </c>
       <c r="AY16" s="13">
         <f t="shared" si="8"/>
-        <v>0.10315471698113195</v>
+        <v>0.1072244897959183</v>
       </c>
       <c r="AZ16" s="4">
         <f t="shared" si="31"/>
-        <v>70.899999999999636</v>
+        <v>68.559999999999491</v>
       </c>
       <c r="BB16" s="8">
         <f t="shared" ref="BB16" si="81">A16</f>
@@ -3995,7 +3995,7 @@
       </c>
       <c r="BF16" s="4">
         <f t="shared" ref="BF16" si="85">(L16-K16)-(L15-K15)</f>
-        <v>4.6800000000000637</v>
+        <v>2.339999999999975</v>
       </c>
       <c r="BG16" s="4">
         <f t="shared" ref="BG16" si="86">(O16-N16)-(O15-N15)</f>
@@ -4053,14 +4053,14 @@
         <v>1.8449999999999998</v>
       </c>
       <c r="K17" s="21">
-        <v>515.39</v>
+        <v>514.99</v>
       </c>
       <c r="L17" s="4">
-        <v>551.17999999999995</v>
+        <v>554.53</v>
       </c>
       <c r="M17" s="12">
         <f t="shared" ref="M17" si="92">(L17-K17)/K17</f>
-        <v>6.9442558062826135E-2</v>
+        <v>7.6778189867764357E-2</v>
       </c>
       <c r="N17" s="5">
         <v>620</v>
@@ -4145,27 +4145,27 @@
       </c>
       <c r="AM17" s="4">
         <f t="shared" si="3"/>
-        <v>1845.3899999999999</v>
+        <v>1844.99</v>
       </c>
       <c r="AN17" s="4">
         <f t="shared" ref="AN17" si="103">AM17-AM16</f>
-        <v>45.389999999999873</v>
+        <v>244.99</v>
       </c>
       <c r="AO17" s="4">
         <f t="shared" si="4"/>
-        <v>2067.35</v>
+        <v>2070.6999999999998</v>
       </c>
       <c r="AP17" s="4">
         <f t="shared" ref="AP17" si="104">AO17-AM17</f>
-        <v>221.96000000000004</v>
+        <v>225.70999999999981</v>
       </c>
       <c r="AQ17" s="13">
         <f t="shared" ref="AQ17" si="105">AP17/AM17</f>
-        <v>0.12027809839654494</v>
+        <v>0.12233670643201308</v>
       </c>
       <c r="AR17" s="4">
         <f t="shared" ref="AR17" si="106">AP17-AP16</f>
-        <v>-6.7799999999999727</v>
+        <v>7.6300000000001091</v>
       </c>
       <c r="AS17" s="10"/>
       <c r="AT17" s="8">
@@ -4174,27 +4174,27 @@
       </c>
       <c r="AU17" s="4">
         <f t="shared" ref="AU17" si="108">AE17+AM17</f>
-        <v>2825.39</v>
+        <v>2824.99</v>
       </c>
       <c r="AV17" s="4">
         <f t="shared" ref="AV17" si="109">AU17-AU16</f>
-        <v>175.38999999999987</v>
+        <v>374.98999999999978</v>
       </c>
       <c r="AW17" s="4">
         <f t="shared" ref="AW17" si="110">AG17+AO17</f>
-        <v>3138.85</v>
+        <v>3142.2</v>
       </c>
       <c r="AX17" s="4">
         <f t="shared" ref="AX17" si="111">AW17-AU17</f>
-        <v>313.46000000000004</v>
+        <v>317.21000000000004</v>
       </c>
       <c r="AY17" s="13">
         <f t="shared" ref="AY17" si="112">AX17/AU17</f>
-        <v>0.1109439758758968</v>
+        <v>0.11228712314025893</v>
       </c>
       <c r="AZ17" s="4">
         <f t="shared" ref="AZ17" si="113">AX17-AX16</f>
-        <v>40.100000000000364</v>
+        <v>54.510000000000218</v>
       </c>
       <c r="BB17" s="8">
         <f t="shared" ref="BB17" si="114">A17</f>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="BF17" s="4">
         <f t="shared" ref="BF17" si="118">(L17-K17)-(L16-K16)</f>
-        <v>-13.450000000000045</v>
+        <v>0.95999999999997954</v>
       </c>
       <c r="BG17" s="4">
         <f t="shared" ref="BG17" si="119">(O17-N17)-(O16-N16)</f>
@@ -4272,14 +4272,14 @@
         <v>1.8449999999999998</v>
       </c>
       <c r="K18" s="21">
-        <v>624.35</v>
+        <v>623.95000000000005</v>
       </c>
       <c r="L18" s="4">
-        <v>663.89</v>
+        <v>663.49</v>
       </c>
       <c r="M18" s="12">
         <f t="shared" ref="M18" si="125">(L18-K18)/K18</f>
-        <v>6.3329863057579816E-2</v>
+        <v>6.3370462376792946E-2</v>
       </c>
       <c r="N18" s="5">
         <v>620</v>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="AM18" s="4">
         <f t="shared" si="3"/>
-        <v>1954.35</v>
+        <v>1953.95</v>
       </c>
       <c r="AN18" s="4">
         <f t="shared" ref="AN18" si="136">AM18-AM17</f>
@@ -4372,19 +4372,19 @@
       </c>
       <c r="AO18" s="4">
         <f t="shared" si="4"/>
-        <v>2191.88</v>
+        <v>2191.48</v>
       </c>
       <c r="AP18" s="4">
         <f t="shared" ref="AP18" si="137">AO18-AM18</f>
-        <v>237.5300000000002</v>
+        <v>237.52999999999997</v>
       </c>
       <c r="AQ18" s="13">
         <f t="shared" ref="AQ18" si="138">AP18/AM18</f>
-        <v>0.12153913065725187</v>
+        <v>0.12156401136160085</v>
       </c>
       <c r="AR18" s="4">
         <f t="shared" ref="AR18" si="139">AP18-AP17</f>
-        <v>15.570000000000164</v>
+        <v>11.820000000000164</v>
       </c>
       <c r="AS18" s="10"/>
       <c r="AT18" s="8">
@@ -4393,7 +4393,7 @@
       </c>
       <c r="AU18" s="4">
         <f t="shared" ref="AU18" si="141">AE18+AM18</f>
-        <v>3064.35</v>
+        <v>3063.95</v>
       </c>
       <c r="AV18" s="4">
         <f t="shared" ref="AV18" si="142">AU18-AU17</f>
@@ -4401,19 +4401,19 @@
       </c>
       <c r="AW18" s="4">
         <f t="shared" ref="AW18" si="143">AG18+AO18</f>
-        <v>3408.4300000000003</v>
+        <v>3408.0299999999997</v>
       </c>
       <c r="AX18" s="4">
         <f t="shared" ref="AX18" si="144">AW18-AU18</f>
-        <v>344.08000000000038</v>
+        <v>344.07999999999993</v>
       </c>
       <c r="AY18" s="13">
         <f t="shared" ref="AY18" si="145">AX18/AU18</f>
-        <v>0.11228482386150419</v>
+        <v>0.11229948269390817</v>
       </c>
       <c r="AZ18" s="4">
         <f t="shared" ref="AZ18" si="146">AX18-AX17</f>
-        <v>30.620000000000346</v>
+        <v>26.869999999999891</v>
       </c>
       <c r="BB18" s="8">
         <f t="shared" ref="BB18" si="147">A18</f>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="BF18" s="4">
         <f t="shared" ref="BF18" si="151">(L18-K18)-(L17-K17)</f>
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="BG18" s="4">
         <f t="shared" ref="BG18" si="152">(O18-N18)-(O17-N17)</f>
@@ -4491,14 +4491,14 @@
         <v>1.8449999999999998</v>
       </c>
       <c r="K19" s="21">
-        <v>624.35</v>
+        <v>623.95000000000005</v>
       </c>
       <c r="L19" s="4">
-        <v>666.13</v>
+        <v>665.73</v>
       </c>
       <c r="M19" s="12">
         <f t="shared" ref="M19" si="158">(L19-K19)/K19</f>
-        <v>6.6917594298069941E-2</v>
+        <v>6.6960493629297166E-2</v>
       </c>
       <c r="N19" s="5">
         <v>620</v>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="AM19" s="4">
         <f>H19+K19+N19+Q19+T19+W19+Z19</f>
-        <v>1954.35</v>
+        <v>1953.95</v>
       </c>
       <c r="AN19" s="4">
         <f t="shared" ref="AN19" si="169">AM19-AM18</f>
@@ -4591,15 +4591,15 @@
       </c>
       <c r="AO19" s="4">
         <f>I19+L19+O19+R19+U19+X19+AA19</f>
-        <v>2199.12</v>
+        <v>2198.7199999999998</v>
       </c>
       <c r="AP19" s="4">
         <f t="shared" ref="AP19" si="170">AO19-AM19</f>
-        <v>244.76999999999998</v>
+        <v>244.76999999999975</v>
       </c>
       <c r="AQ19" s="13">
         <f t="shared" ref="AQ19" si="171">AP19/AM19</f>
-        <v>0.12524368715941361</v>
+        <v>0.12526932623659753</v>
       </c>
       <c r="AR19" s="4">
         <f t="shared" ref="AR19" si="172">AP19-AP18</f>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AU19" s="4">
         <f t="shared" ref="AU19" si="174">AE19+AM19</f>
-        <v>3194.35</v>
+        <v>3193.95</v>
       </c>
       <c r="AV19" s="4">
         <f t="shared" ref="AV19" si="175">AU19-AU18</f>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="AW19" s="4">
         <f t="shared" ref="AW19" si="176">AG19+AO19</f>
-        <v>3536.99</v>
+        <v>3536.5899999999997</v>
       </c>
       <c r="AX19" s="4">
         <f t="shared" ref="AX19" si="177">AW19-AU19</f>
@@ -4628,11 +4628,11 @@
       </c>
       <c r="AY19" s="13">
         <f t="shared" ref="AY19" si="178">AX19/AU19</f>
-        <v>0.10726438868627416</v>
+        <v>0.10727782213246917</v>
       </c>
       <c r="AZ19" s="4">
         <f t="shared" ref="AZ19" si="179">AX19-AX18</f>
-        <v>-1.4400000000005093</v>
+        <v>-1.4400000000000546</v>
       </c>
       <c r="BB19" s="8">
         <f t="shared" ref="BB19" si="180">A19</f>
@@ -4807,7 +4807,7 @@
       </c>
       <c r="AN20" s="4">
         <f t="shared" ref="AN20" si="202">AM20-AM19</f>
-        <v>309.59999999999991</v>
+        <v>309.99999999999977</v>
       </c>
       <c r="AO20" s="4">
         <f>I20+L20+O20+R20+U20+X20+AA20</f>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="AR20" s="4">
         <f t="shared" ref="AR20" si="205">AP20-AP19</f>
-        <v>14.880000000000564</v>
+        <v>14.880000000000791</v>
       </c>
       <c r="AS20" s="10"/>
       <c r="AT20" s="8">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="AV20" s="4">
         <f t="shared" ref="AV20" si="208">AU20-AU19</f>
-        <v>439.59999999999991</v>
+        <v>440</v>
       </c>
       <c r="AW20" s="4">
         <f t="shared" ref="AW20" si="209">AG20+AO20</f>

</xml_diff>

<commit_message>
Dashboard update 2026-10-12 17:46
</commit_message>
<xml_diff>
--- a/excel/Investavimas Rima.xlsx
+++ b/excel/Investavimas Rima.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.08.08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6581A8F-7EAC-4F3D-9925-DCD5BCB07754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{228EB3BC-823C-4A07-8EC4-DE0A9DDEA3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2109,10 +2109,10 @@
         <v>0</v>
       </c>
       <c r="Q8" s="5">
-        <v>410</v>
+        <v>205</v>
       </c>
       <c r="R8" s="4">
-        <v>430</v>
+        <v>215</v>
       </c>
       <c r="S8" s="12">
         <f t="shared" ref="S8:S12" si="36">(R8-Q8)/Q8</f>
@@ -2181,27 +2181,27 @@
       </c>
       <c r="AM8" s="4">
         <f t="shared" si="3"/>
-        <v>640</v>
+        <v>435</v>
       </c>
       <c r="AN8" s="4">
         <f t="shared" si="28"/>
-        <v>610</v>
+        <v>405</v>
       </c>
       <c r="AO8" s="4">
         <f t="shared" si="4"/>
-        <v>715.05</v>
+        <v>500.05</v>
       </c>
       <c r="AP8" s="4">
         <f t="shared" si="5"/>
-        <v>75.049999999999955</v>
+        <v>65.050000000000011</v>
       </c>
       <c r="AQ8" s="13">
         <f t="shared" si="6"/>
-        <v>0.11726562499999993</v>
+        <v>0.1495402298850575</v>
       </c>
       <c r="AR8" s="4">
         <f t="shared" si="29"/>
-        <v>19.999999999999957</v>
+        <v>10.000000000000014</v>
       </c>
       <c r="AS8" s="10"/>
       <c r="AT8" s="8">
@@ -2210,27 +2210,27 @@
       </c>
       <c r="AU8" s="4">
         <f t="shared" si="18"/>
-        <v>850</v>
+        <v>645</v>
       </c>
       <c r="AV8" s="4">
         <f t="shared" si="30"/>
-        <v>640</v>
+        <v>435</v>
       </c>
       <c r="AW8" s="4">
         <f t="shared" si="19"/>
-        <v>929.68</v>
+        <v>714.68000000000006</v>
       </c>
       <c r="AX8" s="4">
         <f t="shared" si="7"/>
-        <v>79.67999999999995</v>
+        <v>69.680000000000064</v>
       </c>
       <c r="AY8" s="13">
         <f t="shared" si="8"/>
-        <v>9.3741176470588175E-2</v>
+        <v>0.10803100775193808</v>
       </c>
       <c r="AZ8" s="4">
         <f t="shared" si="31"/>
-        <v>20.529999999999973</v>
+        <v>10.530000000000086</v>
       </c>
       <c r="BB8" s="8">
         <f t="shared" si="9"/>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="BH8" s="4">
         <f t="shared" si="25"/>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="BI8" s="4">
         <f t="shared" si="32"/>
@@ -2327,10 +2327,10 @@
         <v>4.2499999999999717E-3</v>
       </c>
       <c r="Q9" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R9" s="4">
-        <v>632</v>
+        <v>316</v>
       </c>
       <c r="S9" s="12">
         <f t="shared" si="36"/>
@@ -2399,27 +2399,27 @@
       </c>
       <c r="AM9" s="4">
         <f t="shared" si="3"/>
-        <v>1240</v>
+        <v>935</v>
       </c>
       <c r="AN9" s="4">
         <f t="shared" si="28"/>
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="AO9" s="4">
         <f t="shared" si="4"/>
-        <v>1318.75</v>
+        <v>1002.75</v>
       </c>
       <c r="AP9" s="4">
         <f t="shared" si="5"/>
-        <v>78.75</v>
+        <v>67.75</v>
       </c>
       <c r="AQ9" s="13">
         <f t="shared" si="6"/>
-        <v>6.3508064516129031E-2</v>
+        <v>7.2459893048128346E-2</v>
       </c>
       <c r="AR9" s="4">
         <f t="shared" si="29"/>
-        <v>3.7000000000000455</v>
+        <v>2.6999999999999886</v>
       </c>
       <c r="AS9" s="10"/>
       <c r="AT9" s="8">
@@ -2428,27 +2428,27 @@
       </c>
       <c r="AU9" s="4">
         <f t="shared" si="18"/>
-        <v>1480</v>
+        <v>1175</v>
       </c>
       <c r="AV9" s="4">
         <f t="shared" si="30"/>
-        <v>630</v>
+        <v>530</v>
       </c>
       <c r="AW9" s="4">
         <f t="shared" si="19"/>
-        <v>1564.76</v>
+        <v>1248.76</v>
       </c>
       <c r="AX9" s="4">
         <f t="shared" si="7"/>
-        <v>84.759999999999991</v>
+        <v>73.759999999999991</v>
       </c>
       <c r="AY9" s="13">
         <f t="shared" si="8"/>
-        <v>5.7270270270270263E-2</v>
+        <v>6.277446808510638E-2</v>
       </c>
       <c r="AZ9" s="4">
         <f t="shared" si="31"/>
-        <v>5.0800000000000409</v>
+        <v>4.0799999999999272</v>
       </c>
       <c r="BB9" s="8">
         <f t="shared" si="9"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="BH9" s="4">
         <f t="shared" si="25"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BI9" s="4">
         <f t="shared" si="32"/>
@@ -2545,10 +2545,10 @@
         <v>7.3738095238095297E-2</v>
       </c>
       <c r="Q10" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R10" s="4">
-        <v>634</v>
+        <v>317</v>
       </c>
       <c r="S10" s="12">
         <f t="shared" si="36"/>
@@ -2616,7 +2616,7 @@
       </c>
       <c r="AM10" s="4">
         <f t="shared" si="3"/>
-        <v>1260</v>
+        <v>955</v>
       </c>
       <c r="AN10" s="4">
         <f t="shared" si="28"/>
@@ -2624,19 +2624,19 @@
       </c>
       <c r="AO10" s="4">
         <f t="shared" si="4"/>
-        <v>1370.02</v>
+        <v>1053.02</v>
       </c>
       <c r="AP10" s="4">
         <f t="shared" si="5"/>
-        <v>110.01999999999998</v>
+        <v>98.019999999999982</v>
       </c>
       <c r="AQ10" s="13">
         <f t="shared" si="6"/>
-        <v>8.7317460317460308E-2</v>
+        <v>0.10263874345549737</v>
       </c>
       <c r="AR10" s="4">
         <f t="shared" si="29"/>
-        <v>31.269999999999982</v>
+        <v>30.269999999999982</v>
       </c>
       <c r="AS10" s="10"/>
       <c r="AT10" s="8">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="AU10" s="4">
         <f t="shared" si="18"/>
-        <v>1530</v>
+        <v>1225</v>
       </c>
       <c r="AV10" s="4">
         <f t="shared" si="30"/>
@@ -2653,19 +2653,19 @@
       </c>
       <c r="AW10" s="4">
         <f t="shared" si="19"/>
-        <v>1654.76</v>
+        <v>1337.76</v>
       </c>
       <c r="AX10" s="4">
         <f t="shared" si="7"/>
-        <v>124.75999999999999</v>
+        <v>112.75999999999999</v>
       </c>
       <c r="AY10" s="13">
         <f t="shared" si="8"/>
-        <v>8.1542483660130713E-2</v>
+        <v>9.2048979591836722E-2</v>
       </c>
       <c r="AZ10" s="4">
         <f t="shared" si="31"/>
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="BB10" s="8">
         <f t="shared" si="9"/>
@@ -2693,7 +2693,7 @@
       </c>
       <c r="BH10" s="4">
         <f t="shared" si="25"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BI10" s="4">
         <f t="shared" si="32"/>
@@ -2763,10 +2763,10 @@
         <v>8.6047619047619012E-2</v>
       </c>
       <c r="Q11" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R11" s="4">
-        <v>634</v>
+        <v>317</v>
       </c>
       <c r="S11" s="12">
         <f t="shared" si="36"/>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="AM11" s="4">
         <f t="shared" si="3"/>
-        <v>1360</v>
+        <v>1055</v>
       </c>
       <c r="AN11" s="4">
         <f t="shared" si="28"/>
@@ -2842,15 +2842,15 @@
       </c>
       <c r="AO11" s="4">
         <f t="shared" si="4"/>
-        <v>1500.19</v>
+        <v>1183.19</v>
       </c>
       <c r="AP11" s="4">
         <f t="shared" si="5"/>
-        <v>140.19000000000005</v>
+        <v>128.19000000000005</v>
       </c>
       <c r="AQ11" s="13">
         <f t="shared" si="6"/>
-        <v>0.10308088235294122</v>
+        <v>0.12150710900473939</v>
       </c>
       <c r="AR11" s="4">
         <f t="shared" si="29"/>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="AU11" s="4">
         <f t="shared" si="18"/>
-        <v>1660</v>
+        <v>1355</v>
       </c>
       <c r="AV11" s="4">
         <f t="shared" si="30"/>
@@ -2871,15 +2871,15 @@
       </c>
       <c r="AW11" s="4">
         <f t="shared" si="19"/>
-        <v>1813.3000000000002</v>
+        <v>1496.3000000000002</v>
       </c>
       <c r="AX11" s="4">
         <f t="shared" si="7"/>
-        <v>153.30000000000018</v>
+        <v>141.30000000000018</v>
       </c>
       <c r="AY11" s="13">
         <f t="shared" si="8"/>
-        <v>9.2349397590361551E-2</v>
+        <v>0.10428044280442818</v>
       </c>
       <c r="AZ11" s="4">
         <f t="shared" si="31"/>
@@ -2981,10 +2981,10 @@
         <v>9.6166666666666636E-2</v>
       </c>
       <c r="Q12" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R12" s="4">
-        <v>634</v>
+        <v>317</v>
       </c>
       <c r="S12" s="12">
         <f t="shared" si="36"/>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="AM12" s="4">
         <f t="shared" si="3"/>
-        <v>1360</v>
+        <v>1055</v>
       </c>
       <c r="AN12" s="4">
         <f t="shared" si="28"/>
@@ -3060,15 +3060,15 @@
       </c>
       <c r="AO12" s="4">
         <f t="shared" si="4"/>
-        <v>1510.6100000000001</v>
+        <v>1193.6100000000001</v>
       </c>
       <c r="AP12" s="4">
         <f t="shared" si="5"/>
-        <v>150.61000000000013</v>
+        <v>138.61000000000013</v>
       </c>
       <c r="AQ12" s="13">
         <f t="shared" si="6"/>
-        <v>0.11074264705882363</v>
+        <v>0.13138388625592429</v>
       </c>
       <c r="AR12" s="4">
         <f t="shared" si="29"/>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="AU12" s="4">
         <f t="shared" si="18"/>
-        <v>1660</v>
+        <v>1355</v>
       </c>
       <c r="AV12" s="4">
         <f t="shared" si="30"/>
@@ -3089,15 +3089,15 @@
       </c>
       <c r="AW12" s="4">
         <f t="shared" si="19"/>
-        <v>1828.46</v>
+        <v>1511.46</v>
       </c>
       <c r="AX12" s="4">
         <f t="shared" si="7"/>
-        <v>168.46000000000004</v>
+        <v>156.46000000000004</v>
       </c>
       <c r="AY12" s="13">
         <f t="shared" si="8"/>
-        <v>0.1014819277108434</v>
+        <v>0.1154686346863469</v>
       </c>
       <c r="AZ12" s="4">
         <f t="shared" si="31"/>
@@ -3200,10 +3200,10 @@
         <v>0.10657142857142855</v>
       </c>
       <c r="Q13" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R13" s="4">
-        <v>634</v>
+        <v>317</v>
       </c>
       <c r="S13" s="12">
         <f t="shared" ref="S13" si="46">(R13-Q13)/Q13</f>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="AM13" s="4">
         <f t="shared" si="3"/>
-        <v>1360</v>
+        <v>1055</v>
       </c>
       <c r="AN13" s="4">
         <f t="shared" si="28"/>
@@ -3279,15 +3279,15 @@
       </c>
       <c r="AO13" s="4">
         <f t="shared" si="4"/>
-        <v>1514.98</v>
+        <v>1197.98</v>
       </c>
       <c r="AP13" s="4">
         <f t="shared" si="5"/>
-        <v>154.98000000000002</v>
+        <v>142.98000000000002</v>
       </c>
       <c r="AQ13" s="13">
         <f t="shared" si="6"/>
-        <v>0.11395588235294118</v>
+        <v>0.13552606635071091</v>
       </c>
       <c r="AR13" s="4">
         <f t="shared" si="29"/>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="AU13" s="4">
         <f t="shared" si="18"/>
-        <v>1820</v>
+        <v>1515</v>
       </c>
       <c r="AV13" s="4">
         <f t="shared" si="30"/>
@@ -3308,15 +3308,15 @@
       </c>
       <c r="AW13" s="4">
         <f t="shared" si="19"/>
-        <v>2000.43</v>
+        <v>1683.43</v>
       </c>
       <c r="AX13" s="4">
         <f t="shared" si="7"/>
-        <v>180.43000000000006</v>
+        <v>168.43000000000006</v>
       </c>
       <c r="AY13" s="13">
         <f t="shared" si="8"/>
-        <v>9.9137362637362669E-2</v>
+        <v>0.11117491749174922</v>
       </c>
       <c r="AZ13" s="4">
         <f t="shared" si="31"/>
@@ -3418,10 +3418,10 @@
         <v>0.11692857142857147</v>
       </c>
       <c r="Q14" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R14" s="4">
-        <v>644.72</v>
+        <v>322.36</v>
       </c>
       <c r="S14" s="12">
         <f t="shared" ref="S14" si="52">(R14-Q14)/Q14</f>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="AM14" s="4">
         <f t="shared" si="3"/>
-        <v>1360</v>
+        <v>1055</v>
       </c>
       <c r="AN14" s="4">
         <f t="shared" si="28"/>
@@ -3497,19 +3497,19 @@
       </c>
       <c r="AO14" s="4">
         <f t="shared" si="4"/>
-        <v>1530.0500000000002</v>
+        <v>1207.69</v>
       </c>
       <c r="AP14" s="4">
         <f t="shared" si="5"/>
-        <v>170.05000000000018</v>
+        <v>152.69000000000005</v>
       </c>
       <c r="AQ14" s="13">
         <f t="shared" si="6"/>
-        <v>0.12503676470588249</v>
+        <v>0.14472985781990527</v>
       </c>
       <c r="AR14" s="4">
         <f t="shared" si="29"/>
-        <v>15.070000000000164</v>
+        <v>9.7100000000000364</v>
       </c>
       <c r="AS14" s="10"/>
       <c r="AT14" s="8">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="AU14" s="4">
         <f t="shared" si="18"/>
-        <v>1950</v>
+        <v>1645</v>
       </c>
       <c r="AV14" s="4">
         <f t="shared" si="30"/>
@@ -3526,19 +3526,19 @@
       </c>
       <c r="AW14" s="4">
         <f t="shared" si="19"/>
-        <v>2152.5300000000002</v>
+        <v>1830.17</v>
       </c>
       <c r="AX14" s="4">
         <f t="shared" si="7"/>
-        <v>202.5300000000002</v>
+        <v>185.17000000000007</v>
       </c>
       <c r="AY14" s="13">
         <f t="shared" si="8"/>
-        <v>0.10386153846153856</v>
+        <v>0.11256534954407299</v>
       </c>
       <c r="AZ14" s="4">
         <f t="shared" si="31"/>
-        <v>22.100000000000136</v>
+        <v>16.740000000000009</v>
       </c>
       <c r="BB14" s="8">
         <f t="shared" si="9"/>
@@ -3566,7 +3566,7 @@
       </c>
       <c r="BH14" s="4">
         <f t="shared" si="25"/>
-        <v>10.720000000000027</v>
+        <v>5.3600000000000136</v>
       </c>
       <c r="BI14" s="4">
         <f t="shared" si="32"/>
@@ -3636,10 +3636,10 @@
         <v>9.2629032258064431E-2</v>
       </c>
       <c r="Q15" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R15" s="4">
-        <v>654.46</v>
+        <v>327.23</v>
       </c>
       <c r="S15" s="12">
         <f t="shared" ref="S15" si="58">(R15-Q15)/Q15</f>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="AM15" s="4">
         <f t="shared" si="3"/>
-        <v>1560</v>
+        <v>1255</v>
       </c>
       <c r="AN15" s="4">
         <f t="shared" si="28"/>
@@ -3715,19 +3715,19 @@
       </c>
       <c r="AO15" s="4">
         <f t="shared" si="4"/>
-        <v>1763.23</v>
+        <v>1436</v>
       </c>
       <c r="AP15" s="4">
         <f t="shared" si="5"/>
-        <v>203.23000000000002</v>
+        <v>181</v>
       </c>
       <c r="AQ15" s="13">
         <f t="shared" si="6"/>
-        <v>0.13027564102564104</v>
+        <v>0.14422310756972112</v>
       </c>
       <c r="AR15" s="4">
         <f t="shared" si="29"/>
-        <v>33.179999999999836</v>
+        <v>28.309999999999945</v>
       </c>
       <c r="AS15" s="10"/>
       <c r="AT15" s="8">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="AU15" s="4">
         <f t="shared" si="18"/>
-        <v>2280</v>
+        <v>1975</v>
       </c>
       <c r="AV15" s="4">
         <f t="shared" si="30"/>
@@ -3744,19 +3744,19 @@
       </c>
       <c r="AW15" s="4">
         <f t="shared" si="19"/>
-        <v>2474.1400000000003</v>
+        <v>2146.91</v>
       </c>
       <c r="AX15" s="4">
         <f t="shared" si="7"/>
-        <v>194.14000000000033</v>
+        <v>171.90999999999985</v>
       </c>
       <c r="AY15" s="13">
         <f t="shared" si="8"/>
-        <v>8.5149122807017683E-2</v>
+        <v>8.7043037974683476E-2</v>
       </c>
       <c r="AZ15" s="4">
         <f t="shared" si="31"/>
-        <v>-8.3899999999998727</v>
+        <v>-13.260000000000218</v>
       </c>
       <c r="BB15" s="8">
         <f t="shared" ref="BB15" si="63">A15</f>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="BH15" s="4">
         <f t="shared" ref="BH15" si="69">(R15-Q15)-(R14-Q14)</f>
-        <v>9.7400000000000091</v>
+        <v>4.8700000000000045</v>
       </c>
       <c r="BI15" s="4">
         <f t="shared" si="32"/>
@@ -3854,14 +3854,14 @@
         <v>9.6370967741935487E-2</v>
       </c>
       <c r="Q16" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R16" s="4">
-        <v>664.55</v>
+        <v>332.28</v>
       </c>
       <c r="S16" s="12">
         <f t="shared" ref="S16" si="75">(R16-Q16)/Q16</f>
-        <v>8.9426229508196647E-2</v>
+        <v>8.9442622950819589E-2</v>
       </c>
       <c r="T16" s="5">
         <v>40</v>
@@ -3926,7 +3926,7 @@
       </c>
       <c r="AM16" s="4">
         <f t="shared" si="3"/>
-        <v>1600</v>
+        <v>1295</v>
       </c>
       <c r="AN16" s="4">
         <f t="shared" si="28"/>
@@ -3934,19 +3934,19 @@
       </c>
       <c r="AO16" s="4">
         <f t="shared" si="4"/>
-        <v>1818.0799999999997</v>
+        <v>1485.8099999999997</v>
       </c>
       <c r="AP16" s="4">
         <f t="shared" si="5"/>
-        <v>218.0799999999997</v>
+        <v>190.80999999999972</v>
       </c>
       <c r="AQ16" s="13">
         <f t="shared" si="6"/>
-        <v>0.13629999999999981</v>
+        <v>0.14734362934362913</v>
       </c>
       <c r="AR16" s="4">
         <f t="shared" si="29"/>
-        <v>14.849999999999682</v>
+        <v>9.8099999999997181</v>
       </c>
       <c r="AS16" s="10"/>
       <c r="AT16" s="8">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="AU16" s="4">
         <f t="shared" si="18"/>
-        <v>2450</v>
+        <v>2145</v>
       </c>
       <c r="AV16" s="4">
         <f t="shared" si="30"/>
@@ -3963,19 +3963,19 @@
       </c>
       <c r="AW16" s="4">
         <f t="shared" si="19"/>
-        <v>2712.7</v>
+        <v>2380.4299999999994</v>
       </c>
       <c r="AX16" s="4">
         <f t="shared" si="7"/>
-        <v>262.69999999999982</v>
+        <v>235.42999999999938</v>
       </c>
       <c r="AY16" s="13">
         <f t="shared" si="8"/>
-        <v>0.1072244897959183</v>
+        <v>0.10975757575757547</v>
       </c>
       <c r="AZ16" s="4">
         <f t="shared" si="31"/>
-        <v>68.559999999999491</v>
+        <v>63.519999999999527</v>
       </c>
       <c r="BB16" s="8">
         <f t="shared" ref="BB16" si="81">A16</f>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="BH16" s="4">
         <f t="shared" ref="BH16" si="87">(R16-Q16)-(R15-Q15)</f>
-        <v>10.089999999999918</v>
+        <v>5.0499999999999545</v>
       </c>
       <c r="BI16" s="4">
         <f t="shared" si="32"/>
@@ -4073,14 +4073,14 @@
         <v>0.10343548387096774</v>
       </c>
       <c r="Q17" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R17" s="4">
-        <v>666.19</v>
+        <v>333.1</v>
       </c>
       <c r="S17" s="12">
         <f t="shared" ref="S17" si="94">(R17-Q17)/Q17</f>
-        <v>9.2114754098360743E-2</v>
+        <v>9.2131147540983685E-2</v>
       </c>
       <c r="T17" s="5">
         <v>70</v>
@@ -4145,7 +4145,7 @@
       </c>
       <c r="AM17" s="4">
         <f t="shared" si="3"/>
-        <v>1844.99</v>
+        <v>1539.99</v>
       </c>
       <c r="AN17" s="4">
         <f t="shared" ref="AN17" si="103">AM17-AM16</f>
@@ -4153,19 +4153,19 @@
       </c>
       <c r="AO17" s="4">
         <f t="shared" si="4"/>
-        <v>2070.6999999999998</v>
+        <v>1737.6100000000001</v>
       </c>
       <c r="AP17" s="4">
         <f t="shared" ref="AP17" si="104">AO17-AM17</f>
-        <v>225.70999999999981</v>
+        <v>197.62000000000012</v>
       </c>
       <c r="AQ17" s="13">
         <f t="shared" ref="AQ17" si="105">AP17/AM17</f>
-        <v>0.12233670643201308</v>
+        <v>0.12832550860719882</v>
       </c>
       <c r="AR17" s="4">
         <f t="shared" ref="AR17" si="106">AP17-AP16</f>
-        <v>7.6300000000001091</v>
+        <v>6.8100000000004002</v>
       </c>
       <c r="AS17" s="10"/>
       <c r="AT17" s="8">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="AU17" s="4">
         <f t="shared" ref="AU17" si="108">AE17+AM17</f>
-        <v>2824.99</v>
+        <v>2519.9899999999998</v>
       </c>
       <c r="AV17" s="4">
         <f t="shared" ref="AV17" si="109">AU17-AU16</f>
@@ -4182,19 +4182,19 @@
       </c>
       <c r="AW17" s="4">
         <f t="shared" ref="AW17" si="110">AG17+AO17</f>
-        <v>3142.2</v>
+        <v>2809.11</v>
       </c>
       <c r="AX17" s="4">
         <f t="shared" ref="AX17" si="111">AW17-AU17</f>
-        <v>317.21000000000004</v>
+        <v>289.12000000000035</v>
       </c>
       <c r="AY17" s="13">
         <f t="shared" ref="AY17" si="112">AX17/AU17</f>
-        <v>0.11228712314025893</v>
+        <v>0.11473061401037321</v>
       </c>
       <c r="AZ17" s="4">
         <f t="shared" ref="AZ17" si="113">AX17-AX16</f>
-        <v>54.510000000000218</v>
+        <v>53.690000000000964</v>
       </c>
       <c r="BB17" s="8">
         <f t="shared" ref="BB17" si="114">A17</f>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="BH17" s="4">
         <f t="shared" ref="BH17" si="120">(R17-Q17)-(R16-Q16)</f>
-        <v>1.6400000000001</v>
+        <v>0.82000000000005002</v>
       </c>
       <c r="BI17" s="4">
         <f t="shared" si="32"/>
@@ -4292,10 +4292,10 @@
         <v>0.11838709677419351</v>
       </c>
       <c r="Q18" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R18" s="4">
-        <v>667.84</v>
+        <v>333.92</v>
       </c>
       <c r="S18" s="12">
         <f t="shared" ref="S18" si="127">(R18-Q18)/Q18</f>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="AM18" s="4">
         <f t="shared" si="3"/>
-        <v>1953.95</v>
+        <v>1648.95</v>
       </c>
       <c r="AN18" s="4">
         <f t="shared" ref="AN18" si="136">AM18-AM17</f>
@@ -4372,19 +4372,19 @@
       </c>
       <c r="AO18" s="4">
         <f t="shared" si="4"/>
-        <v>2191.48</v>
+        <v>1857.5600000000002</v>
       </c>
       <c r="AP18" s="4">
         <f t="shared" ref="AP18" si="137">AO18-AM18</f>
-        <v>237.52999999999997</v>
+        <v>208.61000000000013</v>
       </c>
       <c r="AQ18" s="13">
         <f t="shared" ref="AQ18" si="138">AP18/AM18</f>
-        <v>0.12156401136160085</v>
+        <v>0.12651080990933633</v>
       </c>
       <c r="AR18" s="4">
         <f t="shared" ref="AR18" si="139">AP18-AP17</f>
-        <v>11.820000000000164</v>
+        <v>10.990000000000009</v>
       </c>
       <c r="AS18" s="10"/>
       <c r="AT18" s="8">
@@ -4393,7 +4393,7 @@
       </c>
       <c r="AU18" s="4">
         <f t="shared" ref="AU18" si="141">AE18+AM18</f>
-        <v>3063.95</v>
+        <v>2758.95</v>
       </c>
       <c r="AV18" s="4">
         <f t="shared" ref="AV18" si="142">AU18-AU17</f>
@@ -4401,19 +4401,19 @@
       </c>
       <c r="AW18" s="4">
         <f t="shared" ref="AW18" si="143">AG18+AO18</f>
-        <v>3408.0299999999997</v>
+        <v>3074.11</v>
       </c>
       <c r="AX18" s="4">
         <f t="shared" ref="AX18" si="144">AW18-AU18</f>
-        <v>344.07999999999993</v>
+        <v>315.16000000000031</v>
       </c>
       <c r="AY18" s="13">
         <f t="shared" ref="AY18" si="145">AX18/AU18</f>
-        <v>0.11229948269390817</v>
+        <v>0.1142318635712863</v>
       </c>
       <c r="AZ18" s="4">
         <f t="shared" ref="AZ18" si="146">AX18-AX17</f>
-        <v>26.869999999999891</v>
+        <v>26.039999999999964</v>
       </c>
       <c r="BB18" s="8">
         <f t="shared" ref="BB18" si="147">A18</f>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="BH18" s="4">
         <f t="shared" ref="BH18" si="153">(R18-Q18)-(R17-Q17)</f>
-        <v>1.6499999999999773</v>
+        <v>0.81999999999999318</v>
       </c>
       <c r="BI18" s="4">
         <f t="shared" si="32"/>
@@ -4511,10 +4511,10 @@
         <v>0.12248387096774202</v>
       </c>
       <c r="Q19" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R19" s="4">
-        <v>669.6</v>
+        <v>334.8</v>
       </c>
       <c r="S19" s="12">
         <f t="shared" ref="S19" si="160">(R19-Q19)/Q19</f>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="AM19" s="4">
         <f>H19+K19+N19+Q19+T19+W19+Z19</f>
-        <v>1953.95</v>
+        <v>1648.95</v>
       </c>
       <c r="AN19" s="4">
         <f t="shared" ref="AN19" si="169">AM19-AM18</f>
@@ -4591,19 +4591,19 @@
       </c>
       <c r="AO19" s="4">
         <f>I19+L19+O19+R19+U19+X19+AA19</f>
-        <v>2198.7199999999998</v>
+        <v>1863.9199999999998</v>
       </c>
       <c r="AP19" s="4">
         <f t="shared" ref="AP19" si="170">AO19-AM19</f>
-        <v>244.76999999999975</v>
+        <v>214.9699999999998</v>
       </c>
       <c r="AQ19" s="13">
         <f t="shared" ref="AQ19" si="171">AP19/AM19</f>
-        <v>0.12526932623659753</v>
+        <v>0.13036780981836915</v>
       </c>
       <c r="AR19" s="4">
         <f t="shared" ref="AR19" si="172">AP19-AP18</f>
-        <v>7.2399999999997817</v>
+        <v>6.3599999999996726</v>
       </c>
       <c r="AS19" s="10"/>
       <c r="AT19" s="8">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AU19" s="4">
         <f t="shared" ref="AU19" si="174">AE19+AM19</f>
-        <v>3193.95</v>
+        <v>2888.95</v>
       </c>
       <c r="AV19" s="4">
         <f t="shared" ref="AV19" si="175">AU19-AU18</f>
@@ -4620,19 +4620,19 @@
       </c>
       <c r="AW19" s="4">
         <f t="shared" ref="AW19" si="176">AG19+AO19</f>
-        <v>3536.5899999999997</v>
+        <v>3201.79</v>
       </c>
       <c r="AX19" s="4">
         <f t="shared" ref="AX19" si="177">AW19-AU19</f>
-        <v>342.63999999999987</v>
+        <v>312.84000000000015</v>
       </c>
       <c r="AY19" s="13">
         <f t="shared" ref="AY19" si="178">AX19/AU19</f>
-        <v>0.10727782213246917</v>
+        <v>0.10828847851295459</v>
       </c>
       <c r="AZ19" s="4">
         <f t="shared" ref="AZ19" si="179">AX19-AX18</f>
-        <v>-1.4400000000000546</v>
+        <v>-2.3200000000001637</v>
       </c>
       <c r="BB19" s="8">
         <f t="shared" ref="BB19" si="180">A19</f>
@@ -4660,7 +4660,7 @@
       </c>
       <c r="BH19" s="4">
         <f t="shared" ref="BH19" si="186">(R19-Q19)-(R18-Q18)</f>
-        <v>1.7599999999999909</v>
+        <v>0.87999999999999545</v>
       </c>
       <c r="BI19" s="4">
         <f t="shared" si="32"/>
@@ -4730,14 +4730,14 @@
         <v>0.12740322580645164</v>
       </c>
       <c r="Q20" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R20" s="4">
-        <v>678.45</v>
+        <v>339.23</v>
       </c>
       <c r="S20" s="12">
         <f t="shared" ref="S20" si="193">(R20-Q20)/Q20</f>
-        <v>0.11221311475409844</v>
+        <v>0.11222950819672137</v>
       </c>
       <c r="T20" s="5">
         <v>80</v>
@@ -4803,27 +4803,27 @@
       </c>
       <c r="AM20" s="4">
         <f>H20+K20+N20+Q20+T20+W20+Z20</f>
-        <v>2263.9499999999998</v>
+        <v>1958.95</v>
       </c>
       <c r="AN20" s="4">
         <f t="shared" ref="AN20" si="202">AM20-AM19</f>
-        <v>309.99999999999977</v>
+        <v>310</v>
       </c>
       <c r="AO20" s="4">
         <f>I20+L20+O20+R20+U20+X20+AA20</f>
-        <v>2523.6000000000004</v>
+        <v>2184.38</v>
       </c>
       <c r="AP20" s="4">
         <f t="shared" ref="AP20" si="203">AO20-AM20</f>
-        <v>259.65000000000055</v>
+        <v>225.43000000000006</v>
       </c>
       <c r="AQ20" s="13">
         <f t="shared" ref="AQ20" si="204">AP20/AM20</f>
-        <v>0.11468892864241727</v>
+        <v>0.11507695449092629</v>
       </c>
       <c r="AR20" s="4">
         <f t="shared" ref="AR20" si="205">AP20-AP19</f>
-        <v>14.880000000000791</v>
+        <v>10.460000000000264</v>
       </c>
       <c r="AS20" s="10"/>
       <c r="AT20" s="8">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="AU20" s="4">
         <f t="shared" ref="AU20" si="207">AE20+AM20</f>
-        <v>3633.95</v>
+        <v>3328.95</v>
       </c>
       <c r="AV20" s="4">
         <f t="shared" ref="AV20" si="208">AU20-AU19</f>
@@ -4840,19 +4840,19 @@
       </c>
       <c r="AW20" s="4">
         <f t="shared" ref="AW20" si="209">AG20+AO20</f>
-        <v>4021.3</v>
+        <v>3682.08</v>
       </c>
       <c r="AX20" s="4">
         <f t="shared" ref="AX20" si="210">AW20-AU20</f>
-        <v>387.35000000000036</v>
+        <v>353.13000000000011</v>
       </c>
       <c r="AY20" s="13">
         <f t="shared" ref="AY20" si="211">AX20/AU20</f>
-        <v>0.10659200044029235</v>
+        <v>0.10607849321858248</v>
       </c>
       <c r="AZ20" s="4">
         <f t="shared" ref="AZ20" si="212">AX20-AX19</f>
-        <v>44.710000000000491</v>
+        <v>40.289999999999964</v>
       </c>
       <c r="BB20" s="8">
         <f t="shared" ref="BB20" si="213">A20</f>
@@ -4880,7 +4880,7 @@
       </c>
       <c r="BH20" s="4">
         <f t="shared" ref="BH20" si="219">(R20-Q20)-(R19-Q19)</f>
-        <v>8.8500000000000227</v>
+        <v>4.4300000000000068</v>
       </c>
       <c r="BI20" s="4">
         <f t="shared" ref="BI20" si="220">(U20-T20)-(U19-T19)</f>
@@ -4953,14 +4953,14 @@
         <v>0.13695161290322574</v>
       </c>
       <c r="Q21" s="5">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="R21" s="4">
-        <v>687.59</v>
+        <v>343.8</v>
       </c>
       <c r="S21" s="12">
         <f t="shared" ref="S21" si="228">(R21-Q21)/Q21</f>
-        <v>0.12719672131147547</v>
+        <v>0.12721311475409841</v>
       </c>
       <c r="T21" s="5">
         <v>80</v>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="AM21" s="4">
         <f>H21+K21+N21+Q21+T21+W21+Z21</f>
-        <v>2263.9499999999998</v>
+        <v>1958.95</v>
       </c>
       <c r="AN21" s="4">
         <f t="shared" ref="AN21" si="237">AM21-AM20</f>
@@ -5035,19 +5035,19 @@
       </c>
       <c r="AO21" s="4">
         <f>I21+L21+O21+R21+U21+X21+AA21</f>
-        <v>2549.5100000000007</v>
+        <v>2205.7200000000003</v>
       </c>
       <c r="AP21" s="4">
         <f t="shared" ref="AP21" si="238">AO21-AM21</f>
-        <v>285.56000000000085</v>
+        <v>246.77000000000021</v>
       </c>
       <c r="AQ21" s="13">
         <f t="shared" ref="AQ21" si="239">AP21/AM21</f>
-        <v>0.12613352768391567</v>
+        <v>0.12597054544526415</v>
       </c>
       <c r="AR21" s="4">
         <f t="shared" ref="AR21" si="240">AP21-AP20</f>
-        <v>25.910000000000309</v>
+        <v>21.340000000000146</v>
       </c>
       <c r="AS21" s="10"/>
       <c r="AT21" s="8">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="AU21" s="4">
         <f t="shared" ref="AU21" si="242">AE21+AM21</f>
-        <v>3763.95</v>
+        <v>3458.95</v>
       </c>
       <c r="AV21" s="4">
         <f t="shared" ref="AV21" si="243">AU21-AU20</f>
@@ -5064,19 +5064,19 @@
       </c>
       <c r="AW21" s="4">
         <f t="shared" ref="AW21" si="244">AG21+AO21</f>
-        <v>4184.130000000001</v>
+        <v>3840.34</v>
       </c>
       <c r="AX21" s="4">
         <f t="shared" ref="AX21" si="245">AW21-AU21</f>
-        <v>420.1800000000012</v>
+        <v>381.39000000000033</v>
       </c>
       <c r="AY21" s="13">
         <f t="shared" ref="AY21" si="246">AX21/AU21</f>
-        <v>0.11163272625831938</v>
+        <v>0.11026178464562955</v>
       </c>
       <c r="AZ21" s="4">
         <f t="shared" ref="AZ21" si="247">AX21-AX20</f>
-        <v>32.830000000000837</v>
+        <v>28.260000000000218</v>
       </c>
       <c r="BB21" s="8">
         <f t="shared" ref="BB21" si="248">A21</f>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="BH21" s="4">
         <f t="shared" ref="BH21" si="254">(R21-Q21)-(R20-Q20)</f>
-        <v>9.1399999999999864</v>
+        <v>4.5699999999999932</v>
       </c>
       <c r="BI21" s="4">
         <f t="shared" ref="BI21" si="255">(U21-T21)-(U20-T20)</f>

</xml_diff>